<commit_message>
added the image carousel for Rwanda, created new country pages for Colombia, Nepal, Sierra Leone, and Botswana (minus images)
</commit_message>
<xml_diff>
--- a/Books to reference in governance explainer.xlsx
+++ b/Books to reference in governance explainer.xlsx
@@ -384,7 +384,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="39.13" customWidth="1" style="9" min="1" max="1"/>
@@ -1244,6 +1244,141 @@
       <c r="K17" s="12" t="inlineStr">
         <is>
           <t>The central argument inverts modernization theory: political development and economic development are analytically independent, and rapid economic modernization without corresponding institutional development produces not stability but political decay. Huntington argues that the defining challenge for developing societies is building strong, adaptable, autonomous institutions capable of channeling political participation — without them, modernization generates demands that overwhelm political order, producing praetorianism (rule by the military or other non-institutionalized actors). The book's contribution is both a critique of modernization theory's optimism and a framework for understanding political instability in the developing world that remained influential for decades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Why Nations Fail: The Origins of Power, Prosperity, and Poverty</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Acemoglu, Daron; Robinson, James A.</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Crown Business</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Drivers of Democracy, Development, and Rule of Law</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>why-nations-fail.jpg</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Inclusive vs. extractive institutions (Acemoglu &amp; Robinson): inclusive political and economic institutions disperse power, enforce broad property rights, and allow competitive entry; extractive institutions concentrate power and block development. Path dependence through critical junctures. Creative destruction as the mechanism linking inclusive institutions to growth.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>DV: Long-run economic development and political regime type. IVs: Inclusive vs. extractive institutions; distribution of political power; critical historical junctures. Mechanism: inclusive political institutions → inclusive economic institutions → broad investment incentives and creative destruction → growth. Extractive institutions → concentrated rents → blocked entry → stagnation. Virtuous and vicious cycles reinforce each divergence.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Argues that the fundamental cause of poverty is extractive political and economic institutions — not geography, culture, or ignorance. Nations fail because their political systems allow narrow elites to extract wealth from the majority and block the creative destruction that broad growth requires. Inclusive institutions, backed by pluralistic political power, generate the conditions for sustained development. Traces this argument historically across five centuries and dozens of countries. The most widely-cited popular synthesis of the institutions-and-development literature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>The Logic of Political Survival</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Bueno de Mesquita, Bruce; Smith, Alastair; Siverson, Randolph M.; Morrow, James D.</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2003</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MIT Press</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Drivers of Democracy, Development, and Rule of Law</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>the-logic-of-political-survival.jpg</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Selectorate theory: formal game-theoretic model of leader survival based on the size of the winning coalition (W) and the selectorate (S). W/S ratio determines whether private or public goods are the efficient coalition-maintenance strategy. Foundational academic version of what The Dictator's Handbook later popularized.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>DV: Leader survival; policy choices (public vs. private goods provision); economic performance; war initiation; military effectiveness. IVs: Winning coalition size (W); selectorate size (S); W/S ratio. Mechanism: small W → private goods efficient → low public goods investment → poor development outcomes. Large W → private goods too costly → public goods investment → better development outcomes. W/S ratio → interchangeability → coalition bargaining power.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Formal academic statement of selectorate theory: leaders of all regime types are motivated primarily by political survival, and their policy choices are solutions to the coalition-maintenance problem. The key variable is the size of the winning coalition (W) — the minimum group needed to stay in power. Small W makes private payoffs more efficient than public goods, explaining the systematic difference between democracies and autocracies in welfare provision, economic growth, and civil liberties. Tests these predictions empirically across hundreds of country-years. The Logic of Political Survival is the technical foundation; The Dictator's Handbook (2011) is the accessible version of the same argument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rationalist Explanations for War</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fearon, James D.</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1995</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>International Organization, Vol. 49, No. 3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Conflict and Political Violence</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>rationalist-explanations-for-war.jpg</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Bargaining model of war: war as a failure of negotiation between rational actors, driven by three mechanisms — private information with incentives to misrepresent, commitment problems, and issue indivisibility. Foundational framework for rationalist conflict theory.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>DV: War onset and duration. IVs: Private information about capabilities/resolve; commitment problem severity; issue divisibility; presence of enforcement mechanisms. Mechanism: Private information → bluffing → bargaining failure → war. Commitment problem → inability to credibly promise post-deal behavior → preventive or pre-emptive conflict. Issue indivisibility → no compromise available → war. External enforcement reduces commitment problem → enables deals parties cannot reach independently.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Asks why rational actors ever go to war if negotiated settlements would leave both better off. Identifies three rationalist explanations: (1) private information with incentives to misrepresent, preventing identification of mutually preferred deals; (2) commitment problems — inability to credibly promise to honor future agreements even when both sides prefer peace; (3) issue indivisibility, where no compromise is logically available. The commitment problem argument has been especially influential, applied extensively to civil war termination, ethnic conflict, and post-conflict reconstruction. One of the most cited articles in international relations.</t>
         </is>
       </c>
     </row>

</xml_diff>